<commit_message>
another fix to grading
</commit_message>
<xml_diff>
--- a/144/DQ Templates and Instructions/Topic 5 DQ 2/Topic 5 DQ 2.xlsx
+++ b/144/DQ Templates and Instructions/Topic 5 DQ 2/Topic 5 DQ 2.xlsx
@@ -5,12 +5,12 @@
   <workbookPr codeName="ThisWorkbook"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://gcumail-my.sharepoint.com/personal/richard_ketchersid_gcu_edu/Documents/Course Materials/git/Teaching/144/DQ Templates and Instructions/Topic 5 DQ 2/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://gcumail.sharepoint.com/sites/MathematicsProgramFacultyStaff-MATOFTF/Shared Documents/MATOFTF/ALEKS/DQ Templates and Instructions/Topic 5 DQ 2/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="429" documentId="13_ncr:1_{01544684-905C-417E-A831-5CA460CC2737}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{13701FA5-648C-5089-A33E-7230B2E5BF64}"/>
+  <xr:revisionPtr revIDLastSave="437" documentId="13_ncr:1_{01544684-905C-417E-A831-5CA460CC2737}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{EDFBA17D-8293-463C-ACE5-3B8D9698E8AC}"/>
   <bookViews>
-    <workbookView xWindow="1095" yWindow="0" windowWidth="27000" windowHeight="15645" tabRatio="649" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="649" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Goals and Instructions" sheetId="7" r:id="rId1"/>
@@ -6500,7 +6500,7 @@
         <v>#N/A</v>
       </c>
       <c r="K25" s="50" t="b">
-        <f ca="1">IFERROR(OR(J25:J26),FALSE)</f>
+        <f ca="1">IFERROR(OR(J25:J27),FALSE)</f>
         <v>0</v>
       </c>
       <c r="AK25" s="50">
@@ -6545,6 +6545,10 @@
       <c r="F27" s="155"/>
       <c r="G27" s="155"/>
       <c r="H27" s="156"/>
+      <c r="J27" s="50" t="e">
+        <f ca="1">SUBSTITUTE(SUBSTITUTE(_xlfn.FORMULATEXT('Water Quality'!G11), " ",""),"$","") = "=FREQUENCY(Difference_in_water_quality,E11:E20)"</f>
+        <v>#N/A</v>
+      </c>
       <c r="AK27" s="50">
         <f t="shared" si="1"/>
         <v>145</v>
@@ -7765,7 +7769,7 @@
       </c>
     </row>
   </sheetData>
-  <sheetProtection algorithmName="SHA-512" hashValue="YPVebjYUhGbt44GV5/LjJQGkdbY1AOR4VHFZ4fgF19dfIxxpR6wTLej6Al6tJgi8f/Hn23uhiliWkAhDB9UpWA==" saltValue="NqTYqMZdnstkH+c1Vfq59Q==" spinCount="100000" sheet="1" objects="1" scenarios="1"/>
+  <sheetProtection algorithmName="SHA-512" hashValue="B2U0Nw9tFkRrTqNzu4uLjIdeRoY3notrCVZBF0XCAVaZqX1RRmcsY/1RC92isVhdqgWBs0A8o3eyxjxupwGjnQ==" saltValue="ZjDy95YJELmAOjAiI1hydw==" spinCount="100000" sheet="1" objects="1" scenarios="1"/>
   <mergeCells count="9">
     <mergeCell ref="J10:O23"/>
     <mergeCell ref="D24:H27"/>
@@ -18275,121 +18279,121 @@
     <row r="2" spans="1:1">
       <c r="A2" s="3">
         <f ca="1">ROUND(NORMINV(RAND(),68,3.75),1)</f>
-        <v>67.3</v>
+        <v>64.599999999999994</v>
       </c>
     </row>
     <row r="3" spans="1:1">
       <c r="A3" s="3">
         <f t="shared" ref="A3:A66" ca="1" si="0">ROUND(NORMINV(RAND(),68,3.75),1)</f>
-        <v>68.2</v>
+        <v>69.7</v>
       </c>
     </row>
     <row r="4" spans="1:1">
       <c r="A4" s="3">
         <f t="shared" ca="1" si="0"/>
-        <v>67.400000000000006</v>
+        <v>66.900000000000006</v>
       </c>
     </row>
     <row r="5" spans="1:1">
       <c r="A5" s="3">
         <f t="shared" ca="1" si="0"/>
-        <v>70</v>
+        <v>73.5</v>
       </c>
     </row>
     <row r="6" spans="1:1">
       <c r="A6" s="3">
         <f t="shared" ca="1" si="0"/>
-        <v>71.400000000000006</v>
+        <v>68.900000000000006</v>
       </c>
     </row>
     <row r="7" spans="1:1">
       <c r="A7" s="3">
         <f t="shared" ca="1" si="0"/>
-        <v>70.3</v>
+        <v>67.099999999999994</v>
       </c>
     </row>
     <row r="8" spans="1:1">
       <c r="A8" s="3">
         <f t="shared" ca="1" si="0"/>
-        <v>66</v>
+        <v>70.400000000000006</v>
       </c>
     </row>
     <row r="9" spans="1:1">
       <c r="A9" s="3">
         <f t="shared" ca="1" si="0"/>
-        <v>71.599999999999994</v>
+        <v>63.7</v>
       </c>
     </row>
     <row r="10" spans="1:1">
       <c r="A10" s="3">
         <f t="shared" ca="1" si="0"/>
-        <v>64.8</v>
+        <v>73.099999999999994</v>
       </c>
     </row>
     <row r="11" spans="1:1">
       <c r="A11" s="3">
         <f t="shared" ca="1" si="0"/>
-        <v>72.5</v>
+        <v>63.5</v>
       </c>
     </row>
     <row r="12" spans="1:1">
       <c r="A12" s="3">
         <f t="shared" ca="1" si="0"/>
-        <v>73.7</v>
+        <v>67.2</v>
       </c>
     </row>
     <row r="13" spans="1:1">
       <c r="A13" s="3">
         <f t="shared" ca="1" si="0"/>
-        <v>71.400000000000006</v>
+        <v>70.2</v>
       </c>
     </row>
     <row r="14" spans="1:1">
       <c r="A14" s="3">
         <f t="shared" ca="1" si="0"/>
-        <v>63.4</v>
+        <v>74.400000000000006</v>
       </c>
     </row>
     <row r="15" spans="1:1">
       <c r="A15" s="3">
         <f t="shared" ca="1" si="0"/>
-        <v>64.7</v>
+        <v>72.3</v>
       </c>
     </row>
     <row r="16" spans="1:1">
       <c r="A16" s="3">
         <f t="shared" ca="1" si="0"/>
-        <v>69.599999999999994</v>
+        <v>66.400000000000006</v>
       </c>
     </row>
     <row r="17" spans="1:1">
       <c r="A17" s="3">
         <f t="shared" ca="1" si="0"/>
-        <v>65.8</v>
+        <v>69.099999999999994</v>
       </c>
     </row>
     <row r="18" spans="1:1">
       <c r="A18" s="3">
         <f t="shared" ca="1" si="0"/>
-        <v>72.400000000000006</v>
+        <v>62.8</v>
       </c>
     </row>
     <row r="19" spans="1:1">
       <c r="A19" s="3">
         <f t="shared" ca="1" si="0"/>
-        <v>70</v>
+        <v>66.2</v>
       </c>
     </row>
     <row r="20" spans="1:1">
       <c r="A20" s="3">
         <f t="shared" ca="1" si="0"/>
-        <v>69.900000000000006</v>
+        <v>70.5</v>
       </c>
     </row>
     <row r="21" spans="1:1">
       <c r="A21" s="3">
         <f t="shared" ca="1" si="0"/>
-        <v>63.8</v>
+        <v>67.7</v>
       </c>
     </row>
     <row r="22" spans="1:1">
@@ -18401,7 +18405,7 @@
     <row r="23" spans="1:1">
       <c r="A23" s="3">
         <f t="shared" ca="1" si="0"/>
-        <v>65.3</v>
+        <v>62.7</v>
       </c>
     </row>
     <row r="24" spans="1:1">
@@ -18413,7 +18417,7 @@
     <row r="25" spans="1:1">
       <c r="A25" s="3">
         <f t="shared" ca="1" si="0"/>
-        <v>66.099999999999994</v>
+        <v>70.099999999999994</v>
       </c>
     </row>
     <row r="26" spans="1:1">
@@ -18425,331 +18429,331 @@
     <row r="27" spans="1:1">
       <c r="A27" s="3">
         <f t="shared" ca="1" si="0"/>
-        <v>66.3</v>
+        <v>68.7</v>
       </c>
     </row>
     <row r="28" spans="1:1">
       <c r="A28" s="3">
         <f t="shared" ca="1" si="0"/>
-        <v>72.8</v>
+        <v>67.7</v>
       </c>
     </row>
     <row r="29" spans="1:1">
       <c r="A29" s="3">
         <f t="shared" ca="1" si="0"/>
-        <v>70.8</v>
+        <v>75.5</v>
       </c>
     </row>
     <row r="30" spans="1:1">
       <c r="A30" s="3">
         <f t="shared" ca="1" si="0"/>
-        <v>72.2</v>
+        <v>69.900000000000006</v>
       </c>
     </row>
     <row r="31" spans="1:1">
       <c r="A31" s="3">
         <f t="shared" ca="1" si="0"/>
-        <v>69.2</v>
+        <v>67.3</v>
       </c>
     </row>
     <row r="32" spans="1:1">
       <c r="A32" s="3">
         <f t="shared" ca="1" si="0"/>
-        <v>70.099999999999994</v>
+        <v>66.599999999999994</v>
       </c>
     </row>
     <row r="33" spans="1:1">
       <c r="A33" s="3">
         <f t="shared" ca="1" si="0"/>
-        <v>70.2</v>
+        <v>72</v>
       </c>
     </row>
     <row r="34" spans="1:1">
       <c r="A34" s="3">
         <f t="shared" ca="1" si="0"/>
-        <v>62.1</v>
+        <v>73.099999999999994</v>
       </c>
     </row>
     <row r="35" spans="1:1">
       <c r="A35" s="3">
         <f t="shared" ca="1" si="0"/>
-        <v>70.900000000000006</v>
+        <v>64.599999999999994</v>
       </c>
     </row>
     <row r="36" spans="1:1">
       <c r="A36" s="3">
         <f t="shared" ca="1" si="0"/>
-        <v>73.400000000000006</v>
+        <v>64</v>
       </c>
     </row>
     <row r="37" spans="1:1">
       <c r="A37" s="3">
         <f t="shared" ca="1" si="0"/>
-        <v>71.400000000000006</v>
+        <v>79.5</v>
       </c>
     </row>
     <row r="38" spans="1:1">
       <c r="A38" s="3">
         <f t="shared" ca="1" si="0"/>
-        <v>72.5</v>
+        <v>66.099999999999994</v>
       </c>
     </row>
     <row r="39" spans="1:1">
       <c r="A39" s="3">
         <f t="shared" ca="1" si="0"/>
-        <v>65.599999999999994</v>
+        <v>60.2</v>
       </c>
     </row>
     <row r="40" spans="1:1">
       <c r="A40" s="3">
         <f t="shared" ca="1" si="0"/>
-        <v>67.400000000000006</v>
+        <v>58.9</v>
       </c>
     </row>
     <row r="41" spans="1:1">
       <c r="A41" s="3">
         <f t="shared" ca="1" si="0"/>
-        <v>81.8</v>
+        <v>64.2</v>
       </c>
     </row>
     <row r="42" spans="1:1">
       <c r="A42" s="3">
         <f t="shared" ca="1" si="0"/>
-        <v>74.400000000000006</v>
+        <v>73.900000000000006</v>
       </c>
     </row>
     <row r="43" spans="1:1">
       <c r="A43" s="3">
         <f t="shared" ca="1" si="0"/>
-        <v>62.9</v>
+        <v>64.099999999999994</v>
       </c>
     </row>
     <row r="44" spans="1:1">
       <c r="A44" s="3">
         <f t="shared" ca="1" si="0"/>
-        <v>69.3</v>
+        <v>65.599999999999994</v>
       </c>
     </row>
     <row r="45" spans="1:1">
       <c r="A45" s="3">
         <f t="shared" ca="1" si="0"/>
-        <v>71.400000000000006</v>
+        <v>63.2</v>
       </c>
     </row>
     <row r="46" spans="1:1">
       <c r="A46" s="3">
         <f t="shared" ca="1" si="0"/>
-        <v>65.7</v>
+        <v>70</v>
       </c>
     </row>
     <row r="47" spans="1:1">
       <c r="A47" s="3">
         <f t="shared" ca="1" si="0"/>
-        <v>68.400000000000006</v>
+        <v>65.7</v>
       </c>
     </row>
     <row r="48" spans="1:1">
       <c r="A48" s="3">
         <f t="shared" ca="1" si="0"/>
-        <v>63.6</v>
+        <v>70.8</v>
       </c>
     </row>
     <row r="49" spans="1:1">
       <c r="A49" s="3">
         <f t="shared" ca="1" si="0"/>
-        <v>61.7</v>
+        <v>67</v>
       </c>
     </row>
     <row r="50" spans="1:1">
       <c r="A50" s="3">
         <f t="shared" ca="1" si="0"/>
-        <v>66.900000000000006</v>
+        <v>61.5</v>
       </c>
     </row>
     <row r="51" spans="1:1">
       <c r="A51" s="3">
         <f t="shared" ca="1" si="0"/>
-        <v>67.7</v>
+        <v>69</v>
       </c>
     </row>
     <row r="52" spans="1:1">
       <c r="A52" s="3">
         <f t="shared" ca="1" si="0"/>
-        <v>64.099999999999994</v>
+        <v>70.8</v>
       </c>
     </row>
     <row r="53" spans="1:1">
       <c r="A53" s="3">
         <f t="shared" ca="1" si="0"/>
-        <v>66.400000000000006</v>
+        <v>65.7</v>
       </c>
     </row>
     <row r="54" spans="1:1">
       <c r="A54" s="3">
         <f t="shared" ca="1" si="0"/>
-        <v>65.5</v>
+        <v>62.8</v>
       </c>
     </row>
     <row r="55" spans="1:1">
       <c r="A55" s="3">
         <f t="shared" ca="1" si="0"/>
-        <v>63.4</v>
+        <v>69.7</v>
       </c>
     </row>
     <row r="56" spans="1:1">
       <c r="A56" s="3">
         <f t="shared" ca="1" si="0"/>
-        <v>69.099999999999994</v>
+        <v>66.3</v>
       </c>
     </row>
     <row r="57" spans="1:1">
       <c r="A57" s="3">
         <f t="shared" ca="1" si="0"/>
-        <v>66.2</v>
+        <v>67.900000000000006</v>
       </c>
     </row>
     <row r="58" spans="1:1">
       <c r="A58" s="3">
         <f t="shared" ca="1" si="0"/>
-        <v>65.5</v>
+        <v>69.7</v>
       </c>
     </row>
     <row r="59" spans="1:1">
       <c r="A59" s="3">
         <f t="shared" ca="1" si="0"/>
-        <v>69</v>
+        <v>73.7</v>
       </c>
     </row>
     <row r="60" spans="1:1">
       <c r="A60" s="3">
         <f t="shared" ca="1" si="0"/>
-        <v>62</v>
+        <v>71</v>
       </c>
     </row>
     <row r="61" spans="1:1">
       <c r="A61" s="3">
         <f t="shared" ca="1" si="0"/>
-        <v>64.2</v>
+        <v>67.8</v>
       </c>
     </row>
     <row r="62" spans="1:1">
       <c r="A62" s="3">
         <f t="shared" ca="1" si="0"/>
-        <v>67.400000000000006</v>
+        <v>63.9</v>
       </c>
     </row>
     <row r="63" spans="1:1">
       <c r="A63" s="3">
         <f t="shared" ca="1" si="0"/>
-        <v>71.599999999999994</v>
+        <v>65.599999999999994</v>
       </c>
     </row>
     <row r="64" spans="1:1">
       <c r="A64" s="3">
         <f t="shared" ca="1" si="0"/>
-        <v>64.900000000000006</v>
+        <v>70.599999999999994</v>
       </c>
     </row>
     <row r="65" spans="1:1">
       <c r="A65" s="3">
         <f t="shared" ca="1" si="0"/>
-        <v>62.1</v>
+        <v>72.099999999999994</v>
       </c>
     </row>
     <row r="66" spans="1:1">
       <c r="A66" s="3">
         <f t="shared" ca="1" si="0"/>
-        <v>67.900000000000006</v>
+        <v>67.099999999999994</v>
       </c>
     </row>
     <row r="67" spans="1:1">
       <c r="A67" s="3">
         <f t="shared" ref="A67:A103" ca="1" si="1">ROUND(NORMINV(RAND(),68,3.75),1)</f>
-        <v>63.8</v>
+        <v>71.2</v>
       </c>
     </row>
     <row r="68" spans="1:1">
       <c r="A68" s="3">
         <f t="shared" ca="1" si="1"/>
-        <v>73</v>
+        <v>67.7</v>
       </c>
     </row>
     <row r="69" spans="1:1">
       <c r="A69" s="3">
         <f t="shared" ca="1" si="1"/>
-        <v>69.599999999999994</v>
+        <v>71.7</v>
       </c>
     </row>
     <row r="70" spans="1:1">
       <c r="A70" s="3">
         <f t="shared" ca="1" si="1"/>
-        <v>68.5</v>
+        <v>61.6</v>
       </c>
     </row>
     <row r="71" spans="1:1">
       <c r="A71" s="3">
         <f t="shared" ca="1" si="1"/>
-        <v>76.900000000000006</v>
+        <v>72.7</v>
       </c>
     </row>
     <row r="72" spans="1:1">
       <c r="A72" s="3">
         <f t="shared" ca="1" si="1"/>
-        <v>66.400000000000006</v>
+        <v>62.9</v>
       </c>
     </row>
     <row r="73" spans="1:1">
       <c r="A73" s="3">
         <f t="shared" ca="1" si="1"/>
-        <v>71.7</v>
+        <v>68.5</v>
       </c>
     </row>
     <row r="74" spans="1:1">
       <c r="A74" s="3">
         <f t="shared" ca="1" si="1"/>
-        <v>76.400000000000006</v>
+        <v>67.900000000000006</v>
       </c>
     </row>
     <row r="75" spans="1:1">
       <c r="A75" s="3">
         <f t="shared" ca="1" si="1"/>
-        <v>71.3</v>
+        <v>70.7</v>
       </c>
     </row>
     <row r="76" spans="1:1">
       <c r="A76" s="3">
         <f t="shared" ca="1" si="1"/>
-        <v>69.099999999999994</v>
+        <v>61.6</v>
       </c>
     </row>
     <row r="77" spans="1:1">
       <c r="A77" s="3">
         <f t="shared" ca="1" si="1"/>
-        <v>62.2</v>
+        <v>66.8</v>
       </c>
     </row>
     <row r="78" spans="1:1">
       <c r="A78" s="3">
         <f t="shared" ca="1" si="1"/>
-        <v>62.3</v>
+        <v>71.5</v>
       </c>
     </row>
     <row r="79" spans="1:1">
       <c r="A79" s="3">
         <f t="shared" ca="1" si="1"/>
-        <v>70.3</v>
+        <v>68.7</v>
       </c>
     </row>
     <row r="80" spans="1:1">
       <c r="A80" s="3">
         <f t="shared" ca="1" si="1"/>
-        <v>75.8</v>
+        <v>72.2</v>
       </c>
     </row>
     <row r="81" spans="1:1">
       <c r="A81" s="3">
         <f t="shared" ca="1" si="1"/>
-        <v>63.3</v>
+        <v>74.900000000000006</v>
       </c>
     </row>
     <row r="82" spans="1:1">
@@ -18761,127 +18765,127 @@
     <row r="83" spans="1:1">
       <c r="A83" s="3">
         <f t="shared" ca="1" si="1"/>
-        <v>70.099999999999994</v>
+        <v>62.3</v>
       </c>
     </row>
     <row r="84" spans="1:1">
       <c r="A84" s="3">
         <f t="shared" ca="1" si="1"/>
-        <v>71.599999999999994</v>
+        <v>66.5</v>
       </c>
     </row>
     <row r="85" spans="1:1">
       <c r="A85" s="3">
         <f t="shared" ca="1" si="1"/>
-        <v>65.8</v>
+        <v>64.7</v>
       </c>
     </row>
     <row r="86" spans="1:1">
       <c r="A86" s="3">
         <f t="shared" ca="1" si="1"/>
-        <v>67.099999999999994</v>
+        <v>71.099999999999994</v>
       </c>
     </row>
     <row r="87" spans="1:1">
       <c r="A87" s="3">
         <f t="shared" ca="1" si="1"/>
-        <v>66.7</v>
+        <v>71.599999999999994</v>
       </c>
     </row>
     <row r="88" spans="1:1">
       <c r="A88" s="3">
         <f t="shared" ca="1" si="1"/>
-        <v>67.599999999999994</v>
+        <v>74.3</v>
       </c>
     </row>
     <row r="89" spans="1:1">
       <c r="A89" s="3">
         <f t="shared" ca="1" si="1"/>
-        <v>68.8</v>
+        <v>70.900000000000006</v>
       </c>
     </row>
     <row r="90" spans="1:1">
       <c r="A90" s="3">
         <f t="shared" ca="1" si="1"/>
-        <v>67.5</v>
+        <v>62.8</v>
       </c>
     </row>
     <row r="91" spans="1:1">
       <c r="A91" s="3">
         <f t="shared" ca="1" si="1"/>
-        <v>67.900000000000006</v>
+        <v>65.3</v>
       </c>
     </row>
     <row r="92" spans="1:1">
       <c r="A92" s="3">
         <f t="shared" ca="1" si="1"/>
-        <v>66</v>
+        <v>71.599999999999994</v>
       </c>
     </row>
     <row r="93" spans="1:1">
       <c r="A93" s="3">
         <f t="shared" ca="1" si="1"/>
-        <v>66.8</v>
+        <v>67.099999999999994</v>
       </c>
     </row>
     <row r="94" spans="1:1">
       <c r="A94" s="3">
         <f t="shared" ca="1" si="1"/>
-        <v>63.5</v>
+        <v>66.2</v>
       </c>
     </row>
     <row r="95" spans="1:1">
       <c r="A95" s="3">
         <f t="shared" ca="1" si="1"/>
-        <v>67.3</v>
+        <v>67</v>
       </c>
     </row>
     <row r="96" spans="1:1">
       <c r="A96" s="3">
         <f t="shared" ca="1" si="1"/>
-        <v>70.5</v>
+        <v>67.900000000000006</v>
       </c>
     </row>
     <row r="97" spans="1:1">
       <c r="A97" s="3">
         <f t="shared" ca="1" si="1"/>
-        <v>70.2</v>
+        <v>65.400000000000006</v>
       </c>
     </row>
     <row r="98" spans="1:1">
       <c r="A98" s="3">
         <f t="shared" ca="1" si="1"/>
-        <v>74.3</v>
+        <v>65.2</v>
       </c>
     </row>
     <row r="99" spans="1:1">
       <c r="A99" s="3">
         <f t="shared" ca="1" si="1"/>
-        <v>61</v>
+        <v>63.1</v>
       </c>
     </row>
     <row r="100" spans="1:1">
       <c r="A100" s="3">
         <f t="shared" ca="1" si="1"/>
-        <v>61.7</v>
+        <v>66.599999999999994</v>
       </c>
     </row>
     <row r="101" spans="1:1">
       <c r="A101" s="3">
         <f t="shared" ca="1" si="1"/>
-        <v>66.400000000000006</v>
+        <v>65</v>
       </c>
     </row>
     <row r="102" spans="1:1">
       <c r="A102" s="3">
         <f t="shared" ca="1" si="1"/>
-        <v>68.2</v>
+        <v>64.5</v>
       </c>
     </row>
     <row r="103" spans="1:1">
       <c r="A103" s="3">
         <f t="shared" ca="1" si="1"/>
-        <v>72.8</v>
+        <v>68.900000000000006</v>
       </c>
     </row>
   </sheetData>
@@ -18993,6 +18997,16 @@
 </file>
 
 <file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="cca9fd2d-ef84-45c9-8063-8f4bd4c29606">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+  </documentManagement>
+</p:properties>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x0101002C289946819CFF499E91D197BC975371" ma:contentTypeVersion="13" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="674b7a4e239a9748c7aaa97e309327a4">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="cca9fd2d-ef84-45c9-8063-8f4bd4c29606" xmlns:ns3="18557d39-01b8-4d71-9479-3fad465290ae" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="600253478e594d1349e02792803dc53a" ns2:_="" ns3:_="">
     <xsd:import namespace="cca9fd2d-ef84-45c9-8063-8f4bd4c29606"/>
@@ -19209,16 +19223,6 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <lcf76f155ced4ddcb4097134ff3c332f xmlns="cca9fd2d-ef84-45c9-8063-8f4bd4c29606">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </lcf76f155ced4ddcb4097134ff3c332f>
-  </documentManagement>
-</p:properties>
-</file>
-
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{17F1EF20-95AB-4016-A693-6625F3A67214}">
   <ds:schemaRefs>
@@ -19228,6 +19232,16 @@
 </file>
 
 <file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{924A8F3D-57F5-4941-A32A-55B7F7F7AF07}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="cca9fd2d-ef84-45c9-8063-8f4bd4c29606"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{8F527DFD-99D6-4A6C-AC9B-EC23CCFE992B}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -19244,14 +19258,4 @@
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{924A8F3D-57F5-4941-A32A-55B7F7F7AF07}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="cca9fd2d-ef84-45c9-8063-8f4bd4c29606"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
 </file>
</xml_diff>